<commit_message>
AGFEb.CO STD + PP&E + Excel
</commit_message>
<xml_diff>
--- a/data/cox_xlsx/AGFEb.CO.xlsx
+++ b/data/cox_xlsx/AGFEb.CO.xlsx
@@ -8741,13 +8741,34 @@
       <c r="O39" s="16">
         <v>15.06</v>
       </c>
-      <c r="P39" s="15"/>
-      <c r="Q39" s="15"/>
-      <c r="R39" s="15"/>
-      <c r="S39" s="15"/>
-      <c r="T39" s="15"/>
-      <c r="U39" s="15"/>
-      <c r="V39" s="15"/>
+      <c r="P39" s="16">
+        <f t="shared" ref="P39:V39" si="1">P45</f>
+        <v>3.3</v>
+      </c>
+      <c r="Q39" s="16">
+        <f t="shared" si="1"/>
+        <v>8.33</v>
+      </c>
+      <c r="R39" s="16">
+        <f t="shared" si="1"/>
+        <v>10.45</v>
+      </c>
+      <c r="S39" s="16">
+        <f t="shared" si="1"/>
+        <v>7.21</v>
+      </c>
+      <c r="T39" s="16">
+        <f t="shared" si="1"/>
+        <v>7.05</v>
+      </c>
+      <c r="U39" s="16">
+        <f t="shared" si="1"/>
+        <v>7.25</v>
+      </c>
+      <c r="V39" s="16">
+        <f t="shared" si="1"/>
+        <v>6.12</v>
+      </c>
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
@@ -8984,23 +9005,23 @@
         <v>5.29</v>
       </c>
       <c r="P45" s="16">
-        <f t="shared" ref="P45:T45" si="1">SUM(P49:P50)</f>
+        <f t="shared" ref="P45:T45" si="2">SUM(P49:P50)</f>
         <v>3.3</v>
       </c>
       <c r="Q45" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.33</v>
       </c>
       <c r="R45" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10.45</v>
       </c>
       <c r="S45" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.21</v>
       </c>
       <c r="T45" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7.05</v>
       </c>
       <c r="U45" s="16">

</xml_diff>